<commit_message>
Poner el cronograma al dia: siete actividades ya tienen su evidencia en el repositorio
El libro declaraba Pendiente lo que el repositorio ya tiene entregado. Se marcan
Finalizadas las siete actividades cuya evidencia es verificable —los entregables
S19 a S22, la maquina de estados del relevo, la etiqueta de congelacion y las 30
repeticiones en simulacion— y se anota en cada una que artefacto la sostiene.

Los hitos H5 y H7 siguen a las actividades #25 y #37: dejarlos Pendientes ponia al
libro a contradecirse consigo mismo.

Las filas cuyo estado aun depende de una decision —las de hardware bloqueado, las
de la HRI y el acta GO/NO-GO— no se tocan.
</commit_message>
<xml_diff>
--- a/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
+++ b/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
@@ -1253,7 +1253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="B2:C23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="62" min="1" max="1"/>
@@ -1261,7 +1261,6 @@
     <col width="96" customWidth="1" style="62" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="15" customHeight="1" s="63">
       <c r="B2" s="64" t="inlineStr">
         <is>
@@ -1276,7 +1275,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1" s="63">
       <c r="B5" s="66" t="inlineStr">
         <is>
@@ -1425,7 +1423,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="63">
       <c r="B18" s="68" t="inlineStr">
         <is>
@@ -1433,7 +1430,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="25.5" customHeight="1" s="63">
       <c r="B20" s="69" t="inlineStr">
         <is>
@@ -2851,10 +2847,14 @@
       </c>
       <c r="J25" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K25" s="75" t="n"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="K25" s="75" t="inlineStr">
+        <is>
+          <t>Entregado: Entregable_semana_19.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="42.75" customHeight="1" s="63">
       <c r="A26" s="72" t="n">
@@ -2902,12 +2902,12 @@
       </c>
       <c r="J26" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="K26" s="67" t="inlineStr">
         <is>
-          <t>Núcleo del aporte del proyecto; no se recorta. Hito H5</t>
+          <t>Núcleo del aporte del proyecto; no se recorta. Hito H5. Ejecutada y medida el 2026-08-30: S21_relevo_ejecutado.md</t>
         </is>
       </c>
     </row>
@@ -3114,10 +3114,14 @@
       </c>
       <c r="J30" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K30" s="67" t="n"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="K30" s="67" t="inlineStr">
+        <is>
+          <t>Entregado: Entregable_semana_20.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="42.75" customHeight="1" s="63">
       <c r="A31" s="74" t="n">
@@ -3377,10 +3381,14 @@
       </c>
       <c r="J35" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K35" s="75" t="n"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="K35" s="75" t="inlineStr">
+        <is>
+          <t>Entregado: Entregable_semana_21.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1" s="63">
       <c r="A36" s="72" t="n">
@@ -3538,12 +3546,12 @@
       </c>
       <c r="J38" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="K38" s="67" t="inlineStr">
         <is>
-          <t>Hito H7</t>
+          <t>Hito H7. Etiqueta v0.4-implementacion-congelada en el repositorio</t>
         </is>
       </c>
     </row>
@@ -3593,10 +3601,14 @@
       </c>
       <c r="J39" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K39" s="75" t="n"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="K39" s="75" t="inlineStr">
+        <is>
+          <t>Entregado: Entregable_semana_22.tex (la fuente es el entregable versionado)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="42.75" customHeight="1" s="63">
       <c r="A40" s="72" t="n">
@@ -3644,12 +3656,12 @@
       </c>
       <c r="J40" s="78" t="inlineStr">
         <is>
-          <t>Reprogramada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="K40" s="67" t="inlineStr">
         <is>
-          <t>Ejecución de pruebas de evaluación: Cap. 8 S20–S22 → S24–S25. Decisión D1</t>
+          <t>Ejecución de pruebas de evaluación: Cap. 8 S20–S22 → S24–S25. Decisión D1. 30 registros del 2026-09-05 en Documentos/Evidencia/registros</t>
         </is>
       </c>
     </row>
@@ -8573,7 +8585,7 @@
       </c>
       <c r="H6" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizada</t>
         </is>
       </c>
     </row>
@@ -8657,7 +8669,7 @@
       </c>
       <c r="H8" s="77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Finalizada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sin codirectores en todo el repositorio: un solo director, Armando Mateus Rojas
- Portadas de los entregables (.tex y .md, semanas 17 a 28, cronograma S17-S32 y
  actualización del marco) y hoja de cálculo del cronograma: queda solo el director.
- «Los directores» pasa a «el director», con el verbo concordado, en el acta GO/NO-GO, el
  cronograma, los entregables, la evidencia, la bitácora, los planes y guiones de historial
  y el sitio (regenerado).
- La llegada del segundo vehículo y la constancia firmada se cuentan sin atribuir nada a
  los codirectores.
- No se tocan los PDF ya entregados o firmados (anteproyecto, constancia firmada,
  entregables de las semanas 10 a 21): son el registro de lo que se presentó.
</commit_message>
<xml_diff>
--- a/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
+++ b/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C7" s="67" t="inlineStr">
         <is>
-          <t>Ing. Armando Mateus Rojas, Msc. · Ing. Nestor Ivan Ospina, Msc. · Ing. Oscar Mauricio Gélvez Lizarazo, Msc.</t>
+          <t>Ing. Armando Mateus Rojas, Msc.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="K6" s="67" t="inlineStr">
         <is>
-          <t>Constancia de revisión firmada por Armando Mateus el 2026-08-14, dentro del plazo. Firma un solo director, no los tres. D3 y D4 se revisaron el 2026-08-15, después de la firma: se comunican en este corte</t>
+          <t>Constancia de revisión firmada por Armando Mateus el 2026-08-14, dentro del plazo. D3 y D4 se revisaron el 2026-08-15, después de la firma: se comunican en este corte</t>
         </is>
       </c>
     </row>

</xml_diff>